<commit_message>
Aether -> AetherHeaven, epoch 1: cool texels shade on band 0; his cape hangs from the torso
His shader keeps a surface's own hue in shade, where the skin's multiplies
it by a tinted ramp row (warm on 126 / 255, cool on 0). A cool texel on his
pale cloth, between or hair band moves to the skin's 0: Aether10's blue-grey
mane and a lilac cape went peach without it, and moving warm texels too
turned a cream cape lavender and flattened his blonde hair (all in game).

His back cape's top two links per side hang from the skin's upper torso
(50) instead of its back coat chain, whose top links meet at the skin's
centre seam and closed the cape's two panels over the split between them.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/AetherRemapDraft.xlsx
+++ b/Data/RemapDrafts/AetherRemapDraft.xlsx
@@ -1231,14 +1231,14 @@
         <v>42</v>
       </c>
       <c r="B44" t="n">
-        <v>74</v>
+        <v>50</v>
       </c>
       <c r="E44" t="n">
         <v>0.9419999999999999</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Reviewed: root of his left INNER cape chain (42 -&gt; 46 -&gt; 47 -&gt; 49) -&gt; root of the skin's left BACK coat chain (74 -&gt; 76 -&gt; 78 -&gt; 80), height for height. Both his cape chains on a side ride that side's back coat chain, so the two sides move alike. Tool proposed main:100 [136 verts (Body) -&gt; 253 verts (Body), dist 0.1029; runner-up 74 at dist 0.1000; in chain 41-42 -&gt; 99-100]</t>
+          <t>In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 74. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: root of his left INNER cape chain (42 -&gt; 46 -&gt; 47 -&gt; 49) -&gt; root of the skin's left BACK coat chain (74 -&gt; 76 -&gt; 78 -&gt; 80), height for height. Both his cape chains on a side ride that side's back coat chain, so the two sides move alike. Tool proposed main:100 [136 verts (Body) -&gt; 253 verts (Body), dist 0.1029; runner-up 74 at dist 0.1000; in chain 41-42 -&gt; 99-100]</t>
         </is>
       </c>
     </row>
@@ -1247,14 +1247,14 @@
         <v>43</v>
       </c>
       <c r="B45" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="E45" t="n">
         <v>0.977</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Reviewed: root of his right inner cape chain -&gt; root of the skin's right back coat chain (75), the mirror of 42. The tool put it on the skin's BRAID (118). Tool proposed main:118 [137 verts (Body) -&gt; 166 verts (Head), dist 0.0922; runner-up 116 at dist 0.0936]</t>
+          <t>In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 75. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: root of his right inner cape chain -&gt; root of the skin's right back coat chain (75), the mirror of 42. The tool put it on the skin's BRAID (118). Tool proposed main:118 [137 verts (Body) -&gt; 166 verts (Head), dist 0.0922; runner-up 116 at dist 0.0936]</t>
         </is>
       </c>
     </row>
@@ -1263,14 +1263,14 @@
         <v>44</v>
       </c>
       <c r="B46" t="n">
-        <v>74</v>
+        <v>50</v>
       </c>
       <c r="E46" t="n">
         <v>0.192</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Reviewed: root of his left OUTER cape chain (44 -&gt; 45 -&gt; 48 -&gt; 28) -&gt; the skin's left back coat root (74). Tool proposed main:99 [93 verts (Body) -&gt; 253 verts (Body), dist 0.0924; runner-up 100 at dist 0.1291; in chain 44-47 -&gt; 99-102]</t>
+          <t>In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 74. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: root of his left OUTER cape chain (44 -&gt; 45 -&gt; 48 -&gt; 28) -&gt; the skin's left back coat root (74). Tool proposed main:99 [93 verts (Body) -&gt; 253 verts (Body), dist 0.0924; runner-up 100 at dist 0.1291; in chain 44-47 -&gt; 99-102]</t>
         </is>
       </c>
     </row>
@@ -1279,14 +1279,14 @@
         <v>45</v>
       </c>
       <c r="B47" t="n">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="E47" t="n">
         <v>0.272</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Reviewed: second link of his left outer cape chain -&gt; the second link of the skin's left back coat chain (76). The tool's 100 is the one-sided left drape. Tool proposed main:100 [58 verts (Body) -&gt; 253 verts (Body), dist 0.1060; runner-up 101 at dist 0.1267; in chain 44-47 -&gt; 99-102]</t>
+          <t>In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 76. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: second link of his left outer cape chain -&gt; the second link of the skin's left back coat chain (76). The tool's 100 is the one-sided left drape. Tool proposed main:100 [58 verts (Body) -&gt; 253 verts (Body), dist 0.1060; runner-up 101 at dist 0.1267; in chain 44-47 -&gt; 99-102]</t>
         </is>
       </c>
     </row>
@@ -1295,14 +1295,14 @@
         <v>46</v>
       </c>
       <c r="B48" t="n">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="E48" t="n">
         <v>0.503</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Reviewed: second link of his left inner cape chain -&gt; the skin's left back coat link 76 (the tool's 101 is the left drape). Tool proposed main:101 [58 verts (Body) -&gt; 188 verts (Body), dist 0.1228; runner-up 76 at dist 0.1043; in chain 44-47 -&gt; 99-102]</t>
+          <t>In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 76. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: second link of his left inner cape chain -&gt; the skin's left back coat link 76 (the tool's 101 is the left drape). Tool proposed main:101 [58 verts (Body) -&gt; 188 verts (Body), dist 0.1228; runner-up 76 at dist 0.1043; in chain 44-47 -&gt; 99-102]</t>
         </is>
       </c>
     </row>
@@ -1359,14 +1359,14 @@
         <v>50</v>
       </c>
       <c r="B52" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="E52" t="n">
         <v>0.743</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Reviewed: root of his right outer cape chain -&gt; the skin's right back coat root (75), the mirror of 44. [93 verts (Body) -&gt; 599 verts (Body), dist 0.1509; runner-up 67 at dist 0.1693]</t>
+          <t>In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 75. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: root of his right outer cape chain -&gt; the skin's right back coat root (75), the mirror of 44. [93 verts (Body) -&gt; 599 verts (Body), dist 0.1509; runner-up 67 at dist 0.1693]</t>
         </is>
       </c>
     </row>
@@ -1375,14 +1375,14 @@
         <v>51</v>
       </c>
       <c r="B53" t="n">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="E53" t="n">
         <v>0.743</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Reviewed (kept): second link of his right outer cape chain -&gt; the skin's right back coat link 77. [58 verts (Body) -&gt; 188 verts (Body), dist 0.1547; runner-up 69 at dist 0.1530]</t>
+          <t>In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 77. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed (kept): second link of his right outer cape chain -&gt; the skin's right back coat link 77. [58 verts (Body) -&gt; 188 verts (Body), dist 0.1547; runner-up 69 at dist 0.1530]</t>
         </is>
       </c>
     </row>
@@ -1391,14 +1391,14 @@
         <v>52</v>
       </c>
       <c r="B54" t="n">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="E54" t="n">
         <v>0.592</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Reviewed (kept): second link of his right inner cape chain -&gt; the skin's right back coat link 77. [59 verts (Body) -&gt; 188 verts (Body), dist 0.1041; runner-up 117 at dist 0.1114]</t>
+          <t>In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 77. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed (kept): second link of his right inner cape chain -&gt; the skin's right back coat link 77. [59 verts (Body) -&gt; 188 verts (Body), dist 0.1041; runner-up 117 at dist 0.1114]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aether <-> AetherHeaven: cape and back-coat carriers from the second in-game round
Forward: his inner cape roots go back on the skin's back coat chain (74 /
75) and the links between stay on its upper torso -- every link on the chain
closed his cape's split, every top link on the torso opened it far wider
than on his own card; this gives his narrow slit.

Reverse: the skin's centre back panel (its back coat chains, 74-81) rides
his upper torso (11). On his inner cape chains, which part in his idle, it
hung off to his right with its emblem half dark.

aetherHeavenFix.py: --coolHueMargin (taking in neutral whites made
Aether8's white trousers more orange in shade, so the default stays 4).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/AetherRemapDraft.xlsx
+++ b/Data/RemapDrafts/AetherRemapDraft.xlsx
@@ -1231,14 +1231,14 @@
         <v>42</v>
       </c>
       <c r="B44" t="n">
-        <v>50</v>
+        <v>74</v>
       </c>
       <c r="E44" t="n">
         <v>0.9419999999999999</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 74. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: root of his left INNER cape chain (42 -&gt; 46 -&gt; 47 -&gt; 49) -&gt; root of the skin's left BACK coat chain (74 -&gt; 76 -&gt; 78 -&gt; 80), height for height. Both his cape chains on a side ride that side's back coat chain, so the two sides move alike. Tool proposed main:100 [136 verts (Body) -&gt; 253 verts (Body), dist 0.1029; runner-up 74 at dist 0.1000; in chain 41-42 -&gt; 99-100]</t>
+          <t>In game (epoch 2, 2026-10-25): back on the coat chain root; with every top link on the torso the cape opened far wider than on his card. In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 74. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: root of his left INNER cape chain (42 -&gt; 46 -&gt; 47 -&gt; 49) -&gt; root of the skin's left BACK coat chain (74 -&gt; 76 -&gt; 78 -&gt; 80), height for height. Both his cape chains on a side ride that side's back coat chain, so the two sides move alike. Tool proposed main:100 [136 verts (Body) -&gt; 253 verts (Body), dist 0.1029; runner-up 74 at dist 0.1000; in chain 41-42 -&gt; 99-100]</t>
         </is>
       </c>
     </row>
@@ -1247,14 +1247,14 @@
         <v>43</v>
       </c>
       <c r="B45" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="E45" t="n">
         <v>0.977</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 75. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: root of his right inner cape chain -&gt; root of the skin's right back coat chain (75), the mirror of 42. The tool put it on the skin's BRAID (118). Tool proposed main:118 [137 verts (Body) -&gt; 166 verts (Head), dist 0.0922; runner-up 116 at dist 0.0936]</t>
+          <t>In game (epoch 2, 2026-10-25): back on the coat chain root; with every top link on the torso the cape opened far wider than on his card. In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 75. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: root of his right inner cape chain -&gt; root of the skin's right back coat chain (75), the mirror of 42. The tool put it on the skin's BRAID (118). Tool proposed main:118 [137 verts (Body) -&gt; 166 verts (Head), dist 0.0922; runner-up 116 at dist 0.0936]</t>
         </is>
       </c>
     </row>
@@ -3250,14 +3250,14 @@
         <v>74</v>
       </c>
       <c r="B76" t="n">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="C76" t="n">
         <v>0.336</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Behaviour (kept): the skin's back coat chains (74 -&gt; 76 -&gt; 78 -&gt; 80, and 75 -&gt; ... -&gt; 81) ride his INNER cape chains link for link, the inverse of the forward rows: back cloth onto back cloth. [599 verts (Body) -&gt; 136 verts (Body), dist 0.1000; runner-up 17 at dist 0.1197; in chain 74-75 -&gt; 42-43]</t>
+          <t>In game (reverse epoch 1, 2026-10-25): -&gt; his upper torso (11), was 42. The skin's centre back panel rides these two chains; on his inner cape chains, which part in his idle, it hung off to his right with its emblem half dark. Behaviour (kept): the skin's back coat chains (74 -&gt; 76 -&gt; 78 -&gt; 80, and 75 -&gt; ... -&gt; 81) ride his INNER cape chains link for link, the inverse of the forward rows: back cloth onto back cloth. [599 verts (Body) -&gt; 136 verts (Body), dist 0.1000; runner-up 17 at dist 0.1197; in chain 74-75 -&gt; 42-43]</t>
         </is>
       </c>
     </row>
@@ -3266,14 +3266,14 @@
         <v>75</v>
       </c>
       <c r="B77" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="C77" t="n">
         <v>0.24</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>599 verts (Body) -&gt; 137 verts (Body), dist 0.1002; runner-up 44 at dist 0.2035; in chain 74-75 -&gt; 42-43</t>
+          <t>In game (reverse epoch 1, 2026-10-25): -&gt; his upper torso (11), was 43. The skin's centre back panel rides these two chains; on his inner cape chains, which part in his idle, it hung off to his right with its emblem half dark. 599 verts (Body) -&gt; 137 verts (Body), dist 0.1002; runner-up 44 at dist 0.2035; in chain 74-75 -&gt; 42-43</t>
         </is>
       </c>
     </row>
@@ -3282,14 +3282,14 @@
         <v>76</v>
       </c>
       <c r="B78" t="n">
-        <v>46</v>
+        <v>11</v>
       </c>
       <c r="C78" t="n">
         <v>0.39</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Reviewed: second link of the left back coat chain -&gt; his left inner cape link 46 (one chain with 74 -&gt; 42). The tool's 45 is the OUTER chain. Tool proposed 45 [188 verts (Body) -&gt; 58 verts (Body), dist 0.1547; runner-up 46 at dist 0.1043; in chain 76-78 -&gt; 45-47]</t>
+          <t>In game (reverse epoch 1, 2026-10-25): -&gt; his upper torso (11), was 46. The skin's centre back panel rides these two chains; on his inner cape chains, which part in his idle, it hung off to his right with its emblem half dark. Reviewed: second link of the left back coat chain -&gt; his left inner cape link 46 (one chain with 74 -&gt; 42). The tool's 45 is the OUTER chain. Tool proposed 45 [188 verts (Body) -&gt; 58 verts (Body), dist 0.1547; runner-up 46 at dist 0.1043; in chain 76-78 -&gt; 45-47]</t>
         </is>
       </c>
     </row>
@@ -3298,14 +3298,14 @@
         <v>77</v>
       </c>
       <c r="B79" t="n">
-        <v>52</v>
+        <v>11</v>
       </c>
       <c r="C79" t="n">
         <v>0.411</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Reviewed: second link of the RIGHT back coat chain -&gt; his right inner cape link 52. The tool's 46 is on his LEFT side. Tool proposed 46 [188 verts (Body) -&gt; 58 verts (Body), dist 0.1846; runner-up 52 at dist 0.1041; in chain 76-78 -&gt; 45-47]</t>
+          <t>In game (reverse epoch 1, 2026-10-25): -&gt; his upper torso (11), was 52. The skin's centre back panel rides these two chains; on his inner cape chains, which part in his idle, it hung off to his right with its emblem half dark. Reviewed: second link of the RIGHT back coat chain -&gt; his right inner cape link 52. The tool's 46 is on his LEFT side. Tool proposed 46 [188 verts (Body) -&gt; 58 verts (Body), dist 0.1846; runner-up 52 at dist 0.1041; in chain 76-78 -&gt; 45-47]</t>
         </is>
       </c>
     </row>
@@ -3314,14 +3314,14 @@
         <v>78</v>
       </c>
       <c r="B80" t="n">
-        <v>47</v>
+        <v>11</v>
       </c>
       <c r="C80" t="n">
         <v>0.281</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>178 verts (Body) -&gt; 93 verts (Body), dist 0.0771; runner-up 53 at dist 0.1864; in chain 76-78 -&gt; 45-47</t>
+          <t>In game (reverse epoch 1, 2026-10-25): -&gt; his upper torso (11), was 47. The skin's centre back panel rides these two chains; on his inner cape chains, which part in his idle, it hung off to his right with its emblem half dark. 178 verts (Body) -&gt; 93 verts (Body), dist 0.0771; runner-up 53 at dist 0.1864; in chain 76-78 -&gt; 45-47</t>
         </is>
       </c>
     </row>
@@ -3330,14 +3330,14 @@
         <v>79</v>
       </c>
       <c r="B81" t="n">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="C81" t="n">
         <v>0.537</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>178 verts (Body) -&gt; 94 verts (Body), dist 0.0775; runner-up 55 at dist 0.1225</t>
+          <t>In game (reverse epoch 1, 2026-10-25): -&gt; his upper torso (11), was 53. The skin's centre back panel rides these two chains; on his inner cape chains, which part in his idle, it hung off to his right with its emblem half dark. 178 verts (Body) -&gt; 94 verts (Body), dist 0.0775; runner-up 55 at dist 0.1225</t>
         </is>
       </c>
     </row>
@@ -3346,14 +3346,14 @@
         <v>80</v>
       </c>
       <c r="B82" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="C82" t="n">
         <v>0.386</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>114 verts (Body) -&gt; 86 verts (Body), dist 0.0684; runner-up 47 at dist 0.1372</t>
+          <t>In game (reverse epoch 1, 2026-10-25): -&gt; his upper torso (11), was 49. The skin's centre back panel rides these two chains; on his inner cape chains, which part in his idle, it hung off to his right with its emblem half dark. 114 verts (Body) -&gt; 86 verts (Body), dist 0.0684; runner-up 47 at dist 0.1372</t>
         </is>
       </c>
     </row>
@@ -3362,14 +3362,14 @@
         <v>81</v>
       </c>
       <c r="B83" t="n">
-        <v>55</v>
+        <v>11</v>
       </c>
       <c r="C83" t="n">
         <v>0.38</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>114 verts (Body) -&gt; 86 verts (Body), dist 0.0684; runner-up 53 at dist 0.1384</t>
+          <t>In game (reverse epoch 1, 2026-10-25): -&gt; his upper torso (11), was 55. The skin's centre back panel rides these two chains; on his inner cape chains, which part in his idle, it hung off to his right with its emblem half dark. 114 verts (Body) -&gt; 86 verts (Body), dist 0.0684; runner-up 53 at dist 0.1384</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aether <-> AetherHeaven, a share sweep in game: cape 50/50, drape pull 7 cm, side panels 8 cm
Forward: each back-cape link 50% on the skin's back coat chain, 50% on its
torso -- 60/40 left a cloak's slit a hairline (Aether2, Aether3), 40/60
opened the cape wider than his card.

Reverse: the coat's side panels (66-73) are pulled 8 cm in at the hem as
well (on his outer cape chains they flared wider than on the skin; 4 cm
still flared), and with them the drape pull is 7 cm: emblem and pendant
where the original's hang.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/AetherRemapDraft.xlsx
+++ b/Data/RemapDrafts/AetherRemapDraft.xlsx
@@ -998,7 +998,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>In game (epochs 1-4, 2026-10-25): SHARED 70% with the coat chain bone, 30% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. Reviewed (kept): the gold tip of his right outer cape chain -&gt; the skin's lowest right back coat link (81), the mirror of 28 -&gt; 80. [232 verts (Body) -&gt; 114 verts (Body), dist 0.1533; runner-up 73 at dist 0.1884]</t>
+          <t>In game (epochs 1-6 and a share sweep, 2026-10-25): SHARED 50% with the coat chain bone, 50% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. Reviewed (kept): the gold tip of his right outer cape chain -&gt; the skin's lowest right back coat link (81), the mirror of 28 -&gt; 80. [232 verts (Body) -&gt; 114 verts (Body), dist 0.1533; runner-up 73 at dist 0.1884]</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>In game (epochs 1-4, 2026-10-25): SHARED 70% with the coat chain bone, 30% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. Reviewed: the gold TIP of his left outer cape chain (rigid, at y 0.57) -&gt; the skin's lowest left back coat link (80), the end of the same chain. The tool's 103 is the left drape. Tool proposed main:103 [232 verts (Body) -&gt; 108 verts (Body), dist 0.0509; runner-up 80 at dist 0.1533]</t>
+          <t>In game (epochs 1-6 and a share sweep, 2026-10-25): SHARED 50% with the coat chain bone, 50% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. Reviewed: the gold TIP of his left outer cape chain (rigid, at y 0.57) -&gt; the skin's lowest left back coat link (80), the end of the same chain. The tool's 103 is the left drape. Tool proposed main:103 [232 verts (Body) -&gt; 108 verts (Body), dist 0.0509; runner-up 80 at dist 0.1533]</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>In game (epochs 1-4, 2026-10-25): SHARED 70% with the coat chain bone, 30% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. In game (epoch 2, 2026-10-25): back on the coat chain root; with every top link on the torso the cape opened far wider than on his card. In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 74. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: root of his left INNER cape chain (42 -&gt; 46 -&gt; 47 -&gt; 49) -&gt; root of the skin's left BACK coat chain (74 -&gt; 76 -&gt; 78 -&gt; 80), height for height. Both his cape chains on a side ride that side's back coat chain, so the two sides move alike. Tool proposed main:100 [136 verts (Body) -&gt; 253 verts (Body), dist 0.1029; runner-up 74 at dist 0.1000; in chain 41-42 -&gt; 99-100]</t>
+          <t>In game (epochs 1-6 and a share sweep, 2026-10-25): SHARED 50% with the coat chain bone, 50% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. In game (epoch 2, 2026-10-25): back on the coat chain root; with every top link on the torso the cape opened far wider than on his card. In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 74. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: root of his left INNER cape chain (42 -&gt; 46 -&gt; 47 -&gt; 49) -&gt; root of the skin's left BACK coat chain (74 -&gt; 76 -&gt; 78 -&gt; 80), height for height. Both his cape chains on a side ride that side's back coat chain, so the two sides move alike. Tool proposed main:100 [136 verts (Body) -&gt; 253 verts (Body), dist 0.1029; runner-up 74 at dist 0.1000; in chain 41-42 -&gt; 99-100]</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>In game (epochs 1-4, 2026-10-25): SHARED 70% with the coat chain bone, 30% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. In game (epoch 2, 2026-10-25): back on the coat chain root; with every top link on the torso the cape opened far wider than on his card. In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 75. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: root of his right inner cape chain -&gt; root of the skin's right back coat chain (75), the mirror of 42. The tool put it on the skin's BRAID (118). Tool proposed main:118 [137 verts (Body) -&gt; 166 verts (Head), dist 0.0922; runner-up 116 at dist 0.0936]</t>
+          <t>In game (epochs 1-6 and a share sweep, 2026-10-25): SHARED 50% with the coat chain bone, 50% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. In game (epoch 2, 2026-10-25): back on the coat chain root; with every top link on the torso the cape opened far wider than on his card. In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 75. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: root of his right inner cape chain -&gt; root of the skin's right back coat chain (75), the mirror of 42. The tool put it on the skin's BRAID (118). Tool proposed main:118 [137 verts (Body) -&gt; 166 verts (Head), dist 0.0922; runner-up 116 at dist 0.0936]</t>
         </is>
       </c>
     </row>
@@ -1270,7 +1270,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>In game (epochs 1-4, 2026-10-25): SHARED 70% with the coat chain bone, 30% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 74. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: root of his left OUTER cape chain (44 -&gt; 45 -&gt; 48 -&gt; 28) -&gt; the skin's left back coat root (74). Tool proposed main:99 [93 verts (Body) -&gt; 253 verts (Body), dist 0.0924; runner-up 100 at dist 0.1291; in chain 44-47 -&gt; 99-102]</t>
+          <t>In game (epochs 1-6 and a share sweep, 2026-10-25): SHARED 50% with the coat chain bone, 50% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 74. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: root of his left OUTER cape chain (44 -&gt; 45 -&gt; 48 -&gt; 28) -&gt; the skin's left back coat root (74). Tool proposed main:99 [93 verts (Body) -&gt; 253 verts (Body), dist 0.0924; runner-up 100 at dist 0.1291; in chain 44-47 -&gt; 99-102]</t>
         </is>
       </c>
     </row>
@@ -1286,7 +1286,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>In game (epochs 1-4, 2026-10-25): SHARED 70% with the coat chain bone, 30% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 76. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: second link of his left outer cape chain -&gt; the second link of the skin's left back coat chain (76). The tool's 100 is the one-sided left drape. Tool proposed main:100 [58 verts (Body) -&gt; 253 verts (Body), dist 0.1060; runner-up 101 at dist 0.1267; in chain 44-47 -&gt; 99-102]</t>
+          <t>In game (epochs 1-6 and a share sweep, 2026-10-25): SHARED 50% with the coat chain bone, 50% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 76. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: second link of his left outer cape chain -&gt; the second link of the skin's left back coat chain (76). The tool's 100 is the one-sided left drape. Tool proposed main:100 [58 verts (Body) -&gt; 253 verts (Body), dist 0.1060; runner-up 101 at dist 0.1267; in chain 44-47 -&gt; 99-102]</t>
         </is>
       </c>
     </row>
@@ -1302,7 +1302,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>In game (epochs 1-4, 2026-10-25): SHARED 70% with the coat chain bone, 30% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 76. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: second link of his left inner cape chain -&gt; the skin's left back coat link 76 (the tool's 101 is the left drape). Tool proposed main:101 [58 verts (Body) -&gt; 188 verts (Body), dist 0.1228; runner-up 76 at dist 0.1043; in chain 44-47 -&gt; 99-102]</t>
+          <t>In game (epochs 1-6 and a share sweep, 2026-10-25): SHARED 50% with the coat chain bone, 50% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 76. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: second link of his left inner cape chain -&gt; the skin's left back coat link 76 (the tool's 101 is the left drape). Tool proposed main:101 [58 verts (Body) -&gt; 188 verts (Body), dist 0.1228; runner-up 76 at dist 0.1043; in chain 44-47 -&gt; 99-102]</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>In game (epochs 1-4, 2026-10-25): SHARED 70% with the coat chain bone, 30% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. Reviewed: third link of his left inner cape chain -&gt; the skin's left back coat link 78. Tool proposed main:102 [93 verts (Body) -&gt; 180 verts (Body), dist 0.0904; runner-up 101 at dist 0.1273; in chain 44-47 -&gt; 99-102]</t>
+          <t>In game (epochs 1-6 and a share sweep, 2026-10-25): SHARED 50% with the coat chain bone, 50% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. Reviewed: third link of his left inner cape chain -&gt; the skin's left back coat link 78. Tool proposed main:102 [93 verts (Body) -&gt; 180 verts (Body), dist 0.0904; runner-up 101 at dist 0.1273; in chain 44-47 -&gt; 99-102]</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>In game (epochs 1-4, 2026-10-25): SHARED 70% with the coat chain bone, 30% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. Reviewed: third link of his left outer cape chain -&gt; the skin's left back coat link 78. Tool proposed main:102 [93 verts (Body) -&gt; 180 verts (Body), dist 0.0603; runner-up 103 at dist 0.1658; in chain 48-49 -&gt; 102-103]</t>
+          <t>In game (epochs 1-6 and a share sweep, 2026-10-25): SHARED 50% with the coat chain bone, 50% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. Reviewed: third link of his left outer cape chain -&gt; the skin's left back coat link 78. Tool proposed main:102 [93 verts (Body) -&gt; 180 verts (Body), dist 0.0603; runner-up 103 at dist 0.1658; in chain 48-49 -&gt; 102-103]</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>In game (epochs 1-4, 2026-10-25): SHARED 70% with the coat chain bone, 30% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. Reviewed: lowest link of his left inner cape chain -&gt; the lowest link of the skin's left back coat chain (80). Tool proposed main:103 [86 verts (Body) -&gt; 108 verts (Body), dist 0.1130; runner-up 80 at dist 0.0684; in chain 48-49 -&gt; 102-103]</t>
+          <t>In game (epochs 1-6 and a share sweep, 2026-10-25): SHARED 50% with the coat chain bone, 50% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. Reviewed: lowest link of his left inner cape chain -&gt; the lowest link of the skin's left back coat chain (80). Tool proposed main:103 [86 verts (Body) -&gt; 108 verts (Body), dist 0.1130; runner-up 80 at dist 0.0684; in chain 48-49 -&gt; 102-103]</t>
         </is>
       </c>
     </row>
@@ -1366,7 +1366,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>In game (epochs 1-4, 2026-10-25): SHARED 70% with the coat chain bone, 30% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 75. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: root of his right outer cape chain -&gt; the skin's right back coat root (75), the mirror of 44. [93 verts (Body) -&gt; 599 verts (Body), dist 0.1509; runner-up 67 at dist 0.1693]</t>
+          <t>In game (epochs 1-6 and a share sweep, 2026-10-25): SHARED 50% with the coat chain bone, 50% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 75. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed: root of his right outer cape chain -&gt; the skin's right back coat root (75), the mirror of 44. [93 verts (Body) -&gt; 599 verts (Body), dist 0.1509; runner-up 67 at dist 0.1693]</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1382,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>In game (epochs 1-4, 2026-10-25): SHARED 70% with the coat chain bone, 30% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 77. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed (kept): second link of his right outer cape chain -&gt; the skin's right back coat link 77. [58 verts (Body) -&gt; 188 verts (Body), dist 0.1547; runner-up 69 at dist 0.1530]</t>
+          <t>In game (epochs 1-6 and a share sweep, 2026-10-25): SHARED 50% with the coat chain bone, 50% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 77. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed (kept): second link of his right outer cape chain -&gt; the skin's right back coat link 77. [58 verts (Body) -&gt; 188 verts (Body), dist 0.1547; runner-up 69 at dist 0.1530]</t>
         </is>
       </c>
     </row>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>In game (epochs 1-4, 2026-10-25): SHARED 70% with the coat chain bone, 30% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 77. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed (kept): second link of his right inner cape chain -&gt; the skin's right back coat link 77. [59 verts (Body) -&gt; 188 verts (Body), dist 0.1041; runner-up 117 at dist 0.1114]</t>
+          <t>In game (epochs 1-6 and a share sweep, 2026-10-25): SHARED 50% with the coat chain bone, 50% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. In game (epoch 1, 2026-10-25): -&gt; the skin's upper torso (50), was 77. On the back coat chain's top links, which meet at the skin's centre seam, his cape's two panels closed over the split between them; on the torso the split shows as on his own card, and the lower links still swing on the coat chain. Reviewed (kept): second link of his right inner cape chain -&gt; the skin's right back coat link 77. [59 verts (Body) -&gt; 188 verts (Body), dist 0.1041; runner-up 117 at dist 0.1114]</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>In game (epochs 1-4, 2026-10-25): SHARED 70% with the coat chain bone, 30% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. Reviewed (kept): third link of his right inner cape chain -&gt; right back coat link 79. [94 verts (Body) -&gt; 178 verts (Body), dist 0.0775; runner-up 78 at dist 0.1864]</t>
+          <t>In game (epochs 1-6 and a share sweep, 2026-10-25): SHARED 50% with the coat chain bone, 50% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. Reviewed (kept): third link of his right inner cape chain -&gt; right back coat link 79. [94 verts (Body) -&gt; 178 verts (Body), dist 0.0775; runner-up 78 at dist 0.1864]</t>
         </is>
       </c>
     </row>
@@ -1430,7 +1430,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>In game (epochs 1-4, 2026-10-25): SHARED 70% with the coat chain bone, 30% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. Reviewed (kept): third link of his right outer cape chain -&gt; right back coat link 79. [93 verts (Body) -&gt; 178 verts (Body), dist 0.1671; runner-up 71 at dist 0.1453]</t>
+          <t>In game (epochs 1-6 and a share sweep, 2026-10-25): SHARED 50% with the coat chain bone, 50% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. Reviewed (kept): third link of his right outer cape chain -&gt; right back coat link 79. [93 verts (Body) -&gt; 178 verts (Body), dist 0.1671; runner-up 71 at dist 0.1453]</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>In game (epochs 1-4, 2026-10-25): SHARED 70% with the coat chain bone, 30% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. Reviewed (kept): lowest link of his right inner cape chain -&gt; the skin's lowest right back coat link (81). [86 verts (Body) -&gt; 114 verts (Body), dist 0.0684; runner-up 79 at dist 0.1225]</t>
+          <t>In game (epochs 1-6 and a share sweep, 2026-10-25): SHARED 50% with the coat chain bone, 50% the skin's upper torso (50) -- AetherFixer's splitGroups; the row's own value is overridden. Reviewed (kept): lowest link of his right inner cape chain -&gt; the skin's lowest right back coat link (81). [86 verts (Body) -&gt; 114 verts (Body), dist 0.0684; runner-up 79 at dist 0.1225]</t>
         </is>
       </c>
     </row>
@@ -3129,7 +3129,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Behaviour: ROOT of the skin's left SIDE coat panel (66 -&gt; 68 -&gt; 70 -&gt; 72) -&gt; the root of his left OUTER cape chain (44 -&gt; 45 -&gt; 48 -&gt; 28), link for link: hanging cloth onto hanging cloth. His cape hangs ~13 cm behind where the side panel sits, so the panel swings about a pivot behind it -- watch the hips in motion. The tool put this root on his waist (17). Tool proposed 17 [902 verts (Body) -&gt; 538 verts (Body), dist 0.1555; runner-up 42 at dist 0.1882; in chain 66-67 -&gt; 17-18]</t>
+          <t>In game (2026-10-25): also pulled 8 cm in at the hem (AetherHeavenFixer) -- on his outer cape chain it flared wider than on the skin. Behaviour: ROOT of the skin's left SIDE coat panel (66 -&gt; 68 -&gt; 70 -&gt; 72) -&gt; the root of his left OUTER cape chain (44 -&gt; 45 -&gt; 48 -&gt; 28), link for link: hanging cloth onto hanging cloth. His cape hangs ~13 cm behind where the side panel sits, so the panel swings about a pivot behind it -- watch the hips in motion. The tool put this root on his waist (17). Tool proposed 17 [902 verts (Body) -&gt; 538 verts (Body), dist 0.1555; runner-up 42 at dist 0.1882; in chain 66-67 -&gt; 17-18]</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3145,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Reviewed: root of the right side coat panel -&gt; the root of his right outer cape chain (50), the mirror of 66 -&gt; 44. The tool put it on his right UPPER ARM (18): the coat would lift with the arm. Tool proposed 18 [900 verts (Body) -&gt; 321 verts (Body), dist 0.1683; runner-up 43 at dist 0.1883; in chain 66-67 -&gt; 17-18]</t>
+          <t>In game (2026-10-25): also pulled 8 cm in at the hem (AetherHeavenFixer) -- on his outer cape chain it flared wider than on the skin. Reviewed: root of the right side coat panel -&gt; the root of his right outer cape chain (50), the mirror of 66 -&gt; 44. The tool put it on his right UPPER ARM (18): the coat would lift with the arm. Tool proposed 18 [900 verts (Body) -&gt; 321 verts (Body), dist 0.1683; runner-up 43 at dist 0.1883; in chain 66-67 -&gt; 17-18]</t>
         </is>
       </c>
     </row>
@@ -3161,7 +3161,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Behaviour (kept): second link of the left side coat panel -&gt; his left outer cape link 45; see 66. [578 verts (Body) -&gt; 58 verts (Body), dist 0.1530; runner-up 87 at dist 0.1689]</t>
+          <t>In game (2026-10-25): also pulled 8 cm in at the hem (AetherHeavenFixer) -- on his outer cape chain it flared wider than on the skin. Behaviour (kept): second link of the left side coat panel -&gt; his left outer cape link 45; see 66. [578 verts (Body) -&gt; 58 verts (Body), dist 0.1530; runner-up 87 at dist 0.1689]</t>
         </is>
       </c>
     </row>
@@ -3177,7 +3177,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Reviewed (kept): second link of the right side panel -&gt; right outer cape link 51. [578 verts (Body) -&gt; 58 verts (Body), dist 0.1530; runner-up 46 at dist 0.2927]</t>
+          <t>In game (2026-10-25): also pulled 8 cm in at the hem (AetherHeavenFixer) -- on his outer cape chain it flared wider than on the skin. Reviewed (kept): second link of the right side panel -&gt; right outer cape link 51. [578 verts (Body) -&gt; 58 verts (Body), dist 0.1530; runner-up 46 at dist 0.2927]</t>
         </is>
       </c>
     </row>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Reviewed (kept): third link of the left side panel -&gt; his left outer cape link 48. [164 verts (Body) -&gt; 93 verts (Body), dist 0.1453; runner-up 16 at dist 0.2133]</t>
+          <t>In game (2026-10-25): also pulled 8 cm in at the hem (AetherHeavenFixer) -- on his outer cape chain it flared wider than on the skin. Reviewed (kept): third link of the left side panel -&gt; his left outer cape link 48. [164 verts (Body) -&gt; 93 verts (Body), dist 0.1453; runner-up 16 at dist 0.2133]</t>
         </is>
       </c>
     </row>
@@ -3209,7 +3209,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Reviewed: third link of the right side panel -&gt; his right outer cape link 54, the mirror of 70 -&gt; 48. The tool's 27 is the chain's end. Tool proposed 27 [164 verts (Body) -&gt; 232 verts (Body), dist 0.2105; runner-up 54 at dist 0.1453; in chain 71-72 -&gt; 27-28]</t>
+          <t>In game (2026-10-25): also pulled 8 cm in at the hem (AetherHeavenFixer) -- on his outer cape chain it flared wider than on the skin. Reviewed: third link of the right side panel -&gt; his right outer cape link 54, the mirror of 70 -&gt; 48. The tool's 27 is the chain's end. Tool proposed 27 [164 verts (Body) -&gt; 232 verts (Body), dist 0.2105; runner-up 54 at dist 0.1453; in chain 71-72 -&gt; 27-28]</t>
         </is>
       </c>
     </row>
@@ -3225,7 +3225,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Reviewed (kept): hem of the left side panel -&gt; the end of his left outer cape chain (28). [116 verts (Body) -&gt; 232 verts (Body), dist 0.1884; runner-up 16 at dist 0.2272; in chain 71-72 -&gt; 27-28]</t>
+          <t>In game (2026-10-25): also pulled 8 cm in at the hem (AetherHeavenFixer) -- on his outer cape chain it flared wider than on the skin. Reviewed (kept): hem of the left side panel -&gt; the end of his left outer cape chain (28). [116 verts (Body) -&gt; 232 verts (Body), dist 0.1884; runner-up 16 at dist 0.2272; in chain 71-72 -&gt; 27-28]</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Reviewed (kept): hem of the right side panel -&gt; the end of his right outer cape chain (27). [116 verts (Body) -&gt; 232 verts (Body), dist 0.1884; runner-up 54 at dist 0.2037]</t>
+          <t>In game (2026-10-25): also pulled 8 cm in at the hem (AetherHeavenFixer) -- on his outer cape chain it flared wider than on the skin. Reviewed (kept): hem of the right side panel -&gt; the end of his right outer cape chain (27). [116 verts (Body) -&gt; 232 verts (Body), dist 0.1884; runner-up 54 at dist 0.2037]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
AetherRemapDraft: his eyes onto the skin's main head, as VGRemapData
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/AetherRemapDraft.xlsx
+++ b/Data/RemapDrafts/AetherRemapDraft.xlsx
@@ -558,15 +558,15 @@
       <c r="A2" t="n">
         <v>0</v>
       </c>
-      <c r="D2" t="n">
-        <v>1</v>
+      <c r="B2" t="n">
+        <v>4</v>
       </c>
       <c r="E2" t="n">
         <v>0.438</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>120 verts (Head) -&gt; 200 verts (A), dist 0.0016; runner-up Bang:1 at dist 0.0612</t>
+          <t>Reviewed (forward epoch 8): his EYE -&gt; the skin's main head (4), not its Eye component: the skin's Eye shader drew an elemental eye mod's glowing iris white / grey, the main mesh glows it as on his card; ordinary eyes unchanged in game. Tool proposed Eye:1 [120 verts (Head) -&gt; 200 verts (A), dist 0.0016; runner-up Bang:1 at dist 0.0612]</t>
         </is>
       </c>
     </row>
@@ -574,15 +574,15 @@
       <c r="A3" t="n">
         <v>1</v>
       </c>
-      <c r="D3" t="n">
-        <v>0</v>
+      <c r="B3" t="n">
+        <v>4</v>
       </c>
       <c r="E3" t="n">
         <v>0.463</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>120 verts (Head) -&gt; 200 verts (A), dist 0.0016; runner-up Bang:2 at dist 0.0451</t>
+          <t>Reviewed (forward epoch 8): his EYE -&gt; the skin's main head (4), not its Eye component: the skin's Eye shader drew an elemental eye mod's glowing iris white / grey, the main mesh glows it as on his card; ordinary eyes unchanged in game. Tool proposed Eye:0 [120 verts (Head) -&gt; 200 verts (A), dist 0.0016; runner-up Bang:2 at dist 0.0451]</t>
         </is>
       </c>
     </row>

</xml_diff>